<commit_message>
V.2 Stakeholders CheerClick Systems
</commit_message>
<xml_diff>
--- a/Documentación/Trimestre I/Stakeholders_CheerClick_Systems.xlsx
+++ b/Documentación/Trimestre I/Stakeholders_CheerClick_Systems.xlsx
@@ -4,10 +4,10 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="Roles" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Gestion de usuarios" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Gestión de Elementos Deportivos" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="Gestión de Horarios" sheetId="4" r:id="rId8"/>
-    <sheet state="visible" name="Gestión de Rendimiento Deportiv" sheetId="5" r:id="rId9"/>
+    <sheet state="visible" name="Gestión de Usuarios" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="Gestión de Horarios" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="Gestión de Rendimiento Deportiv" sheetId="4" r:id="rId8"/>
+    <sheet state="visible" name="Gestión de Elementos Deportivos" sheetId="5" r:id="rId9"/>
     <sheet state="visible" name="Gestión de PQRS" sheetId="6" r:id="rId10"/>
   </sheets>
   <definedNames/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="53">
   <si>
     <t>SISTEMA DE INFORMACIÓN CHEERCLICK SYSTEMS</t>
   </si>
@@ -97,17 +97,24 @@
     <t>Prioridad</t>
   </si>
   <si>
-    <t>Gestion de usuarios</t>
+    <t>Gestion de Horarios</t>
   </si>
   <si>
     <t>Se requiere un módulo centralizado donde se gestione el ciclo de vida de los usuarios dentro de la plataforma, permitiendo el registro de nuevos atletas mediante un formato de captura de datos de contacto para establecer una comunicación efectiva y asegurar su correcta integración en la base de datos. Este componente debe garantizar la seguridad mediante un sistema de autenticación robusto y permitir la gestión de perfiles personalizados.. Asimismo, el sistema debe contemplar la administración de roles y el control de acceso robusto, asegurando que cada usuario interactúe únicamente con las funcionalidades permitidas según su nivel de autorización.
 De acuerdo con los estándares de recolección de información que mencionas, el formulario de registro base para los atletas debe contener los siguientes campos obligatorios:
-- Estado: Activo Inactivo
+- Estado: Activo/Inactivo
 - Nombre completo
 - Número y tipo de documento
+- Edad
+- Genero
+- Telefono
+- Telefono (Acudiente)
+- Fecha de nacimiento
+- Categoría
 - Email
-- Constraseña
-- Certificado de la EPS</t>
+- Contraseña
+- Certificado de la EPS
+- Parentesco</t>
   </si>
   <si>
     <t>Alta</t>
@@ -130,11 +137,13 @@
 El sistema debe permitir a los usuarios un cambio de contraseña en caso de que sea requerido.
 RF - 007 Actualizar Datos del Usuario
 El sistema debe permitir a los usuarios actualizar su información personal registrada
-RF- 008 Administración de Cuentas 
+RF - 008 Edición de Perfil de Usuario
+ El sistema debe permitir al administrador, atleta y entrenador editar la información de su perfil personal, incluyendo datos de contacto, información de emergencia, preferencias de comunicación y contraseña, garantizando la seguridad y actualización correcta de los datos registrados en el sistema.
+RF- 009 Administración de Cuentas 
 El sistema debe permitir al administrador modificar, activar o desactivar cuentas de usuarios.
-RF- 009 Consulta y Registro de Estado de  Mensualidades
+RF- 010 Consulta y Registro de Estado de  Mensualidades
 El sistema debe permitir al administrador registrar y actualizar el estado de las mensualidades de los atletas indicando su respectivo estado con el envío de      notificaciones relacionadas.
-RF- 010 Cierre de Sesión
+RF- 011 Cierre de Sesión
 El sistema debe permitir a los usuarios cerrar sesión de manera segura, finalizando su acceso a la plataforma.
 </t>
   </si>
@@ -146,78 +155,6 @@
   </si>
   <si>
     <t xml:space="preserve">Fecha de especificación </t>
-  </si>
-  <si>
-    <t xml:space="preserve">     Firma                                                                  Firma(s)        Firma(s)
-     ( Dueño del proceso )                                         Usuarios participantes                                      Demás usuarios involucrados
-     en la especificación                                             en la especificación
-</t>
-  </si>
-  <si>
-    <t>Gestión de Elementos Deportivos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El sistema debe permitir el registro y control centralizado de los elementos deportivos del club. Se requiere una gestión eficiente de las solicitudes de préstamo y un seguimiento preciso de la disponibilidad de los recursos para los entrenamientos.
-El sistema debe gestionar los siguientes campos:
-Nombre del elemento
-Cantidad en stock
-Estado (Cliente: Pendiente/Cancelar/Listo para Entregar), (Administrador: Pendiente/Disponible/No Disponible/Rechazado/Aprobado)
-Usuario solicitante
-Fecha de solicitud
-Fecha de entrega
-Productos solicitados
-</t>
-  </si>
-  <si>
-    <t>Controles y Restrcciones o Requerimientos no Funcionales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RF - 015  Registro de Rendimiento Deportivo
-El sistema debe permitir al entrenador evaluar y registrar el desempeño deportivo del atleta, incluyendo evaluaciones de desempeño, mientras que la asistencia será gestionada mediante los registros correspondientes del sistema.
-RF - 016 Consulta de Rendimiento Deportivo
-El sistema debe permitir a los usuarios autorizados consultar el rendimiento deportivo del atleta, incluyendo historial de evaluaciones y registro de asistencia.
-RF - 017  Actualización del Rendimiento Deportivo
-El sistema debe permitir al entrenador modificar registros de rendimiento deportivo, incluyendo evaluaciones y asistencia.
-RF - 018 Inhabilitar  Registro de Rendimiento 
-El sistema debe permitir Inhabilitar registros de evaluaciones o asistencia en caso de errores o duplicados.
-RF-019 – Registro de Asistencia
- El sistema debe permitir al entrenador registrar la asistencia de los atletas a entrenamientos o eventos, filtrando por fecha o categoría y marcando el estado de cada participante (asistió, falta, justificado).
-RF - 020 Justificación de Inasistencia 
-El sistema debe permitir a los clientes justificar la ausencia antes o después de la sesión de entrenamiento programada en su horario.  
-</t>
-  </si>
-  <si>
-    <t>Criterios de Aceptación</t>
-  </si>
-  <si>
-    <t>El sistema debe validar los permisos de usuario en cada transacción de modificación o eliminación. Los registros deben tener integridad referencial para evitar inconsistencias en el historial del atleta. El tiempo de respuesta del sistema para consultas de historial no debe superar los 2 segundos.</t>
-  </si>
-  <si>
-    <t>Fecha de Especifícación</t>
-  </si>
-  <si>
-    <t>Gestion de Horarios</t>
-  </si>
-  <si>
-    <t>Se requiere un módulo para la gestión de cronogramas donde el administrador configure las jornadas de entrenamiento y eventos para posteriormente generar una planificación de los horaios en la base de datos que permitirá establecer una organización eficiente del tiempo.
-- El sistema debe cumplir con las siguientes funciones y registros:
-- Configuración de días y franjas horarias por categoría y nivel
-- Validación automática de disponibilidad de espacio (evitar cruces)
-- Control administrativo para la modificación o inhabilitación de horarios
-- Sistema de notificaciones automáticas para usuarios afectados por cambios</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RF- 011 Definición de Cronograma 
-El sistema debe permitir al administrador configurar los días y franjas horarias de entrenamiento para cada categoría y nivel, verificando que no existan coincidencias en el uso de espacio
-RF- 012 Consultar Horarios
-El sistema debe generar un calendario para cada categoría, filtrando únicamente las sesiones de entrenamiento y eventos que correspondan a cada usuario.
-RF - 013 Modificación de Horarios
-El sistema debe permitir exclusivamente al administrador modificar o inhabilitar los horarios de entrenamiento y torneos previamente definidos, asegurando la consistencia del cronograma y evitando conflictos de programación. Asimismo, el sistema deberá notificar automáticamente a los usuarios afectados por los cambios realizados.
-.
-</t>
-  </si>
-  <si>
-    <t>Para garantizar el correcto funcionamiento del sistema debe validar que el usuario haya sido autenticado previamente con el rol de administrador para realizar cualquier configuración, modificación o Inhabilitación de horarios. El sistema debe asegurar la integridad de la información validando que no existan conflictos o cruces con otros eventos registrados antes de guardar los cambios exitosamente. Asimismo, se debe garantizar la privacidad y relevancia de la información, permitiendo que cada usuario visualice únicamente el calendario y las sesiones que correspondan a su categoría específica.</t>
   </si>
   <si>
     <t xml:space="preserve">     Firma                                                                  Firma(s)        Firma(s)
@@ -226,33 +163,64 @@
 </t>
   </si>
   <si>
+    <t>Se requiere un módulo para la gestión de cronogramas donde el administrador configure las jornadas de entrenamiento y eventos para posteriormente generar una planificación de los horaios en la base de datos que permitirá establecer una organización eficiente del tiempo.
+- El sistema debe cumplir con las siguientes funciones y registros:
+- Consultar Horarios (Atleta, Entrenador)
+- Configuración de días y franjas horarias por categoría y nivel
+- Validación automática de disponibilidad de espacio (evitar cruces)
+- Control administrativo para la modificación o inhabilitación de horarios
+- Sistema de notificaciones automáticas para usuarios afectados por cambios
+- Agregar Nuevo nivel con sus respectivo entrenador y dias de entrenamiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RF- 012 Definición de Cronograma 
+El sistema debe permitir al administrador configurar los días y franjas horarias de entrenamiento para cada categoría y nivel, verificando que no existan coincidencias en el uso de espacio
+RF- 013 Consultar Horarios
+El sistema debe generar un calendario para cada categoría, filtrando únicamente las sesiones de entrenamiento y eventos que correspondan a cada usuario.
+RF - 014 Modificación de Horarios
+El sistema debe permitir exclusivamente al administrador modificar o inhabilitar los horarios de entrenamiento y torneos previamente definidos, asegurando la consistencia del cronograma y evitando conflictos de programación. Asimismo, el sistema deberá notificar automáticamente a los usuarios afectados por los cambios realizados.
+.RF - 015 Registro de Nueva Categoría
+El sistema debe permitir exclusivamente al administrador registrar una nueva categoría deportiva, asignándole un entrenador responsable y definiendo su franja horaria, incluyendo los días de entrenamiento. 
+RF - 016 Inhabilitación de horarios 
+El sistema debe permitir exclusivamente al administrador inhabilitar horarios de entrenamiento previamente definidos, evitando su uso en la programación activa sin eliminarlos del sistema, con el fin de mantener el historial y la integridad de la información. Asimismo, el sistema deberá actualizar automáticamente la disponibilidad y reflejar los cambios en la planificación de las categorías afectadas. 
+</t>
+  </si>
+  <si>
+    <t>Para garantizar el correcto funcionamiento del sistema debe validar que el usuario haya sido autenticado previamente con el rol de administrador para realizar cualquier configuración, modificación o Inhabilitación de horarios. El sistema debe asegurar la integridad de la información validando que no existan conflictos o cruces con otros eventos registrados antes de guardar los cambios exitosamente. Asimismo, se debe garantizar la privacidad y relevancia de la información, permitiendo que cada usuario visualice únicamente el calendario y las sesiones que correspondan a su categoría específica.</t>
+  </si>
+  <si>
     <t>Gestión de Rendimiento Deportivo</t>
   </si>
   <si>
-    <t>El sistema permitirá registrar, monitorear y controlar el rendimietno deportivo de los atletas, basandose en la evaluación del desempeño de los mismos y el seguimiento de asistencia a sesiones de entrenamiento o a eventos.
+    <t xml:space="preserve">El sistema permitirá registrar, monitorear y controlar el rendimietno deportivo de los atletas, basandose en la evaluación del desempeño de los mismos y el seguimiento de asistencia a sesiones de entrenamiento o a eventos.
 Por otra parte el sistema permitirá realizar la justificación de inasistencias de los usuarios, con el fin de llevar un fácil seguimiento de cada uno de los registros e historial deportivo de cada atleta.
 El sistema permitirá gestionar los siguientes campos:
-- Atleta, entrenador encargado
-- Fecha de evaluación
+-  Entrenador encargado del nivel
+- Historial de rendimiento
+- Registrar nuevo desempeño del atleta (Ej: Arcos, Palomas, Fliflas, Mortales) las metricas depende del nivel
+- Consultar rendimiento del atleta
+- Editar rendimeinto del atleta
 - Calificación del desempeño
-- Registro de asistencia (Asistió / Falta / Justificado)
+- Inhabilitar rendimiento del atleta
+- Registro de asistencia (Presente/ Inpuntual / Falta / Justificado)
 - Fecha de asistencia
 - Justificación de la inasistencia
-- Historial de rendimiento</t>
-  </si>
-  <si>
-    <t>RF - 015 Registro de Rendimiento Deportivo
-El sistema debe permitir al entrenador evaluar y registrar el desempeño deportivo del atleta.
-RF - 016 Consulta de Rendimiento Deportivo
-El sistema debe permitir a los usuarios autorizados consultar el rendimiento deportivo del atleta.
-RF - 017 Actualización del Rendimiento Deportivo
-El sistema debe permitir al entrenador modificar registros de rendimiento deportivo.
-RF - 018 Inhabilitar Registro de Rendimiento
-El sistema debe permitir inhabilitar registros de evaluaciones o asistencia en caso de errores o duplicados.
-RF - 019 Registro de Asistencia
-El sistema debe permitir al entrenador registrar la asistencia de los atletas.
-RF - 020 Justificación de Inasistencia
-El sistema debe permitir a los clientes justificar la ausencia a entrenamientos o eventos.</t>
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RF - 017  Registro de Rendimiento Deportivo
+El sistema debe permitir al entrenador evaluar y registrar el desempeño deportivo del atleta, incluyendo evaluaciones de desempeño, mientras que la asistencia será gestionada mediante los registros correspondientes del sistema.
+RF - 018 Consulta de Rendimiento Deportivo
+El sistema debe permitir a los usuarios autorizados consultar el rendimiento deportivo del atleta, incluyendo historial de evaluaciones y registro de asistencia.
+RF - 019  Actualización del Rendimiento Deportivo
+El sistema debe permitir al entrenador modificar registros de rendimiento deportivo, incluyendo evaluaciones y asistencia
+RF - 020 Inhabilitar  Registro de Rendimiento 
+El sistema debe permitir Inhabilitar registros de evaluaciones o asistencia en caso de errores o duplicados.
+RF-021 – Registro de Asistencia
+ El sistema debe permitir al entrenador registrar la asistencia de los atletas a entrenamientos o eventos, filtrando por fecha o categoría y marcando el estado de cada participante (asistió, falta, justificado)
+RF - 022 Justificación de Inasistencia 
+El sistema debe permitir a los clientes justificar la ausencia antes o después de la sesión de entrenamiento programada en su horario.
+</t>
   </si>
   <si>
     <t xml:space="preserve">- Solo el entrenador podrá ingresar los registros de los atletas asignados a él.
@@ -263,36 +231,97 @@
 </t>
   </si>
   <si>
+    <t>Gestión de Elementos Deportivos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El sistema debe permitir el registro y control centralizado de los elementos deportivos del club. Se requiere una gestión eficiente de las solicitudes de préstamo y un seguimiento preciso de la disponibilidad de los recursos para los entrenamientos.
+El sistema debe gestionar los siguientes campos:
+Filtros de Busqueda
+Selección de pestaña: Implementos Deportivos/Productos Solicitados
+Nombre del Implemento
+Tipo de implemento
+Cantidad en stock
+Modificar Implemento deportivo
+Inhabilitar inplemento deportivo
+Precio del implemento
+Solicitud de pedido
+Estado (Cliente: Pendiente/Cancelar/Listo para Entregar), (Administrador: Disponible/No Disponible/Pendiente/Rechazado/Aprobado)
+Nombre del solicitante
+Fecha de solicitud
+Fecha de entrega
+</t>
+  </si>
+  <si>
+    <t>Controles y Restrcciones o Requerimientos no Funcionales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RF - 023 Registro de Implementos Deportivos
+El sistema debe permitir registrar los elementos deportivos, incluyendo nombre del elemento, tipo, precio, observaciones, cantidad disponible y estado.
+RF - 024 Solicitud de Implementos Deportivos
+El sistema debe permitir que los clientes soliciten elementos deportivos para los entrenamientos y competencias.
+RF - 025 Aprobación de Solicitudes de Implementos
+El sistema debe permitir al administrador aprobar o rechazar las solicitudes de implementos deportivos realizadas por los usuarios.
+RF - 026 Consultar Implementos deportivos
+El sistema debe permitir al administrador y a los atletas consultar el listado de implementos deportivos registrados, mostrando información detallada como nombre del implemento, cantidad disponible, estado, categoría.
+RF - 027 Consulta de Productos Solicitados 
+El sistema debe permitir al administrador y al cliente consultar el listado de productos solicitados, mostrando información detallada como el nombre del producto, cantidad, estado de la solicitud, fecha de registro y responsable. 
+RF - 028 Actualización de Implementos
+El sistema debe permitir modificar la información de los implementos deportivos registrados.
+RF - 029 Cancelación  o Inhabilitación de Implementos
+El sistema debe permitir cancelar o inhabilitar implementos deportivos del sistema cuando el cliente quiera cancelarlo, ya no estén disponibles o se hayan discontinuado
+</t>
+  </si>
+  <si>
+    <t>Criterios de Aceptación</t>
+  </si>
+  <si>
+    <t>El sistema debe validar los permisos de usuario en cada transacción de modificación o eliminación. Los registros deben tener integridad referencial para evitar inconsistencias en el historial del atleta. El tiempo de respuesta del sistema para consultas de historial no debe superar los 2 segundos.</t>
+  </si>
+  <si>
+    <t>Fecha de Especifícación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Firma                                                                  Firma(s)        Firma(s)
+     ( Dueño del proceso )                                         Usuarios participantes                                      Demás usuarios involucrados
+     en la especificación                                             en la especificación
+</t>
+  </si>
+  <si>
     <t>Gestión de PQRS</t>
   </si>
   <si>
     <t xml:space="preserve">El sistema debe permitir la gestión integrada de las solicitudes, quejas, reclamos y sugerencias (PQRS) dentro de la platafomra, facilitando a los usuarios el registro, la consulta y asimismo el seguimiento de sus solicitudes.
 También debera garantizar la trazabilidad de cada solicitud mediante la generación automática de un número único, la actualización de su estado y el registro de las respuestas proporcionadas por el administrador.
 El sistema debe gestionar los siguiente campos:
-- Tipo de solicitud (Solicitud, Queja, Reclamo, Sugerencia)
+- Consultar PQRS
+- Registrar tipo de solicitud (Solicitud, Queja, Reclamo, Sugerencia)
 - Número de radicado
 - Descripción
 - Usuario Solicitante
 - Fecha de creación
 - Respuesta del administrador con fecha correspondiente
+- Notificar Respuesta de PQRS
 - Estado de PQRS (pendiente, en trámite y resuelta).
+- Modificar PQRS
+- Inhabilitar PQRS
 </t>
   </si>
   <si>
-    <t>RF - 027 Registro de PQRS
+    <t xml:space="preserve">RF- 030 Registro de PQRS
 El sistema debe permitir a los usuarios registrar peticiones, quejas, reclamos o sugerencias dentro de la plataforma.
-RF - 028 Generación de Radicado
+RF- 031 Generación de Radicado
 El sistema debe asignar automáticamente un número de radicado único a cada solicitud registrada.
-RF - 029 Consulta de PQRS
+RF- 032 Consulta de PQRS
 El sistema debe permitir a los usuarios consultar información relacionada a las solicitudes registradas.
-RF - 030 Actualización de Registro de PQRS
+RF- 033  Actualización de Registro de PQRS
 El sistema debe permitir actualizar el estado y la información relacionada a una solicitud.
-RF - 031 Respuesta de PQRS
+RF- 034 Respuesta de PQRS
 El sistema debe permitir al administrador gestionar y responder las solicitudes registradas.
-RF - 032 Notificación de Estado de PQRS
+RF-035 Notificación de Estado de PQRS
 El sistema debe notificar al usuario cuando su solicitud haya sido respondida.
-RF - 033 Inhabilitación de PQRS
-El sistema debe permitir al administrador inhabilitar solicitudes cuando sea necesario.</t>
+RF - 036 Inhabilitación de PQRS
+El sistema debe permitir al administrador inhabilitar solicitudes de PQRS cuando sea necesario.
+</t>
   </si>
   <si>
     <t>- El sistema debe validar los permisos del usuario para cada proceso (creación, consulta, actualización e inhabilitación).
@@ -441,7 +470,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -478,8 +507,8 @@
     <xf borderId="7" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="7" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
@@ -500,17 +529,14 @@
       <alignment horizontal="left" readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="7" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="7" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -536,7 +562,7 @@
     <xdr:ext cx="1028700" cy="1038225"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -564,7 +590,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -612,19 +638,19 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>4048125</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>142875</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>971550</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2238375" cy="9525"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
+      <xdr:rowOff>495300</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2305050" cy="647700"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -643,40 +669,12 @@
       <xdr:col>3</xdr:col>
       <xdr:colOff>1762125</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>381000</xdr:rowOff>
+      <xdr:rowOff>419100</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1733550" cy="1295400"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>476250</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2305050" cy="647700"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image6.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -702,158 +700,130 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
+      <xdr:colOff>400050</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1028700" cy="1038225"/>
     <xdr:pic>
       <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>180975</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>971550</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2238375" cy="9525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1514475</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>971550</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2238375" cy="9525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>142875</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>495300</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2305050" cy="647700"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1762125</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>419100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1733550" cy="1295400"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
         <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>95250</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>590550</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2238375" cy="9525"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1676400</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>600075</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2238375" cy="9525"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>4314825</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>600075</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2238375" cy="9525"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>66675</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>66675</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2305050" cy="647700"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image6.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1847850</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>581025</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1733550" cy="1295400"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
+        <a:blip cstate="print" r:embed="rId5"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -882,39 +852,11 @@
     <xdr:ext cx="1028700" cy="1038225"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2238375" cy="9525"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -938,7 +880,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -987,14 +929,14 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>142875</xdr:colOff>
+      <xdr:colOff>228600</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>495300</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2305050" cy="647700"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image6.png" title="Imagen"/>
+    <xdr:ext cx="2019300" cy="571500"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1017,16 +959,44 @@
       <xdr:col>3</xdr:col>
       <xdr:colOff>1762125</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>419100</xdr:rowOff>
+      <xdr:rowOff>352425</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1733550" cy="1295400"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>4057650</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>971550</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2238375" cy="9525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1048,158 +1018,158 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>400050</xdr:colOff>
+      <xdr:colOff>190500</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1028700" cy="1038225"/>
     <xdr:pic>
       <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>590550</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2238375" cy="9525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1676400</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>600075</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2238375" cy="9525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>4314825</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>600075</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2238375" cy="9525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2305050" cy="647700"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1847850</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>581025</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1733550" cy="1295400"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
         <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>180975</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>971550</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2238375" cy="9525"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1514475</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>971550</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2238375" cy="9525"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>228600</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>495300</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2019300" cy="571500"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image6.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
         <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1762125</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>352425</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1733550" cy="1295400"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>4057650</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>971550</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2238375" cy="9525"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1228,7 +1198,7 @@
     <xdr:ext cx="1028700" cy="1038225"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1256,7 +1226,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1284,7 +1254,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1312,7 +1282,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1335,12 +1305,12 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>257175</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
+      <xdr:rowOff>133350</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1914525" cy="542925"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image6.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1361,14 +1331,14 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1943100</xdr:colOff>
+      <xdr:colOff>1933575</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>590550</xdr:rowOff>
+      <xdr:rowOff>571500</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1733550" cy="1295400"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1728,8 +1698,10 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" ht="272.25" customHeight="1">
-      <c r="B4" s="14"/>
+    <row r="4" ht="358.5" customHeight="1">
+      <c r="B4" s="14">
+        <v>3.0</v>
+      </c>
       <c r="C4" s="15" t="s">
         <v>25</v>
       </c>
@@ -1740,7 +1712,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" ht="411.0" customHeight="1">
+    <row r="5" ht="476.25" customHeight="1">
       <c r="B5" s="17"/>
       <c r="C5" s="18" t="s">
         <v>28</v>
@@ -1798,80 +1770,80 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="2" max="2" width="8.13"/>
-    <col customWidth="1" min="3" max="3" width="13.63"/>
-    <col customWidth="1" min="4" max="4" width="63.0"/>
-    <col customWidth="1" min="5" max="5" width="23.38"/>
+    <col customWidth="1" min="3" max="3" width="16.0"/>
+    <col customWidth="1" min="4" max="4" width="55.63"/>
+    <col customWidth="1" min="5" max="5" width="27.75"/>
   </cols>
   <sheetData>
-    <row r="2" ht="84.75" customHeight="1">
+    <row r="2" ht="89.25" customHeight="1">
       <c r="B2" s="11"/>
       <c r="C2" s="12"/>
-      <c r="D2" s="24" t="s">
+      <c r="D2" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="24" t="s">
+      <c r="E2" s="13" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" ht="21.75" customHeight="1">
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="D3" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="24" t="s">
+      <c r="E3" s="13" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="4" ht="194.25" customHeight="1">
+    <row r="4" ht="195.0" customHeight="1">
       <c r="B4" s="14">
-        <v>2.0</v>
-      </c>
-      <c r="C4" s="18" t="s">
+        <v>3.0</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="25" t="s">
-        <v>35</v>
-      </c>
       <c r="E4" s="15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" ht="294.0" customHeight="1">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" ht="246.75" customHeight="1">
       <c r="B5" s="17"/>
       <c r="C5" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D5" s="20" t="s">
-        <v>37</v>
+        <v>28</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>35</v>
       </c>
       <c r="E5" s="12"/>
     </row>
-    <row r="6" ht="50.25" customHeight="1">
+    <row r="6" ht="106.5" customHeight="1">
       <c r="B6" s="17"/>
       <c r="C6" s="18" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E6" s="12"/>
     </row>
-    <row r="7" ht="26.25" customHeight="1">
+    <row r="7" ht="36.0" customHeight="1">
       <c r="B7" s="17"/>
       <c r="C7" s="18" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="D7" s="21">
         <v>46136.0</v>
       </c>
       <c r="E7" s="12"/>
     </row>
-    <row r="8" ht="109.5" customHeight="1">
+    <row r="8" ht="144.75" customHeight="1">
       <c r="B8" s="17"/>
       <c r="C8" s="22" t="s">
         <v>33</v>
@@ -1928,37 +1900,37 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" ht="138.0" customHeight="1">
+    <row r="4" ht="296.25" customHeight="1">
       <c r="B4" s="14">
-        <v>3.0</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="D4" s="26" t="s">
-        <v>42</v>
+        <v>4.0</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="24" t="s">
+        <v>38</v>
       </c>
       <c r="E4" s="15" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" ht="142.5" customHeight="1">
+    <row r="5" ht="291.0" customHeight="1">
       <c r="B5" s="17"/>
       <c r="C5" s="18" t="s">
         <v>28</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E5" s="12"/>
     </row>
-    <row r="6" ht="106.5" customHeight="1">
+    <row r="6" ht="91.5" customHeight="1">
       <c r="B6" s="17"/>
       <c r="C6" s="18" t="s">
         <v>30</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="E6" s="12"/>
     </row>
@@ -1975,7 +1947,7 @@
     <row r="8" ht="144.75" customHeight="1">
       <c r="B8" s="17"/>
       <c r="C8" s="22" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="D8" s="23"/>
       <c r="E8" s="12"/>
@@ -2000,83 +1972,83 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="2" max="2" width="8.13"/>
-    <col customWidth="1" min="3" max="3" width="16.0"/>
-    <col customWidth="1" min="4" max="4" width="55.63"/>
-    <col customWidth="1" min="5" max="5" width="27.75"/>
+    <col customWidth="1" min="3" max="3" width="13.63"/>
+    <col customWidth="1" min="4" max="4" width="63.0"/>
+    <col customWidth="1" min="5" max="5" width="23.38"/>
   </cols>
   <sheetData>
-    <row r="2" ht="89.25" customHeight="1">
+    <row r="2" ht="84.75" customHeight="1">
       <c r="B2" s="11"/>
       <c r="C2" s="12"/>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="25" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" ht="21.75" customHeight="1">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="25" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="4" ht="217.5" customHeight="1">
+    <row r="4" ht="263.25" customHeight="1">
       <c r="B4" s="14">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" s="27" t="s">
-        <v>47</v>
+        <v>41</v>
+      </c>
+      <c r="D4" s="26" t="s">
+        <v>42</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" ht="226.5" customHeight="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" ht="360.0" customHeight="1">
       <c r="B5" s="17"/>
       <c r="C5" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="19" t="s">
-        <v>48</v>
+        <v>43</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>44</v>
       </c>
       <c r="E5" s="12"/>
     </row>
-    <row r="6" ht="91.5" customHeight="1">
+    <row r="6" ht="50.25" customHeight="1">
       <c r="B6" s="17"/>
       <c r="C6" s="18" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E6" s="12"/>
     </row>
-    <row r="7" ht="36.0" customHeight="1">
+    <row r="7" ht="26.25" customHeight="1">
       <c r="B7" s="17"/>
       <c r="C7" s="18" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="D7" s="21">
         <v>46136.0</v>
       </c>
       <c r="E7" s="12"/>
     </row>
-    <row r="8" ht="144.75" customHeight="1">
+    <row r="8" ht="109.5" customHeight="1">
       <c r="B8" s="17"/>
       <c r="C8" s="22" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D8" s="23"/>
       <c r="E8" s="12"/>
@@ -2109,65 +2081,65 @@
     <row r="2" ht="84.75" customHeight="1">
       <c r="B2" s="11"/>
       <c r="C2" s="12"/>
-      <c r="D2" s="24" t="s">
+      <c r="D2" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="24" t="s">
+      <c r="E2" s="25" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" ht="21.75" customHeight="1">
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="D3" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="24" t="s">
+      <c r="E3" s="25" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="4" ht="207.0" customHeight="1">
+    <row r="4" ht="270.75" customHeight="1">
       <c r="B4" s="14">
         <v>5.0</v>
       </c>
       <c r="C4" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="26" t="s">
         <v>50</v>
-      </c>
-      <c r="D4" s="25" t="s">
-        <v>51</v>
       </c>
       <c r="E4" s="15" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" ht="257.25" customHeight="1">
+    <row r="5" ht="283.5" customHeight="1">
       <c r="B5" s="17"/>
       <c r="C5" s="18" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E5" s="12"/>
     </row>
     <row r="6" ht="50.25" customHeight="1">
       <c r="B6" s="17"/>
       <c r="C6" s="18" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E6" s="12"/>
     </row>
     <row r="7" ht="26.25" customHeight="1">
       <c r="B7" s="17"/>
       <c r="C7" s="18" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="D7" s="21">
         <v>46136.0</v>
@@ -2177,7 +2149,7 @@
     <row r="8" ht="109.5" customHeight="1">
       <c r="B8" s="17"/>
       <c r="C8" s="22" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="D8" s="23"/>
       <c r="E8" s="12"/>

</xml_diff>

<commit_message>
V.3 Stakeholders CheerClick Systems
</commit_message>
<xml_diff>
--- a/Documentación/Trimestre I/Stakeholders_CheerClick_Systems.xlsx
+++ b/Documentación/Trimestre I/Stakeholders_CheerClick_Systems.xlsx
@@ -7,7 +7,7 @@
     <sheet state="visible" name="Gestión de Usuarios" sheetId="2" r:id="rId6"/>
     <sheet state="visible" name="Gestión de Horarios" sheetId="3" r:id="rId7"/>
     <sheet state="visible" name="Gestión de Rendimiento Deportiv" sheetId="4" r:id="rId8"/>
-    <sheet state="visible" name="Gestión de Elementos Deportivos" sheetId="5" r:id="rId9"/>
+    <sheet state="visible" name="Gestión de Implementos Deportiv" sheetId="5" r:id="rId9"/>
     <sheet state="visible" name="Gestión de PQRS" sheetId="6" r:id="rId10"/>
   </sheets>
   <definedNames/>
@@ -231,7 +231,7 @@
 </t>
   </si>
   <si>
-    <t>Gestión de Elementos Deportivos</t>
+    <t>Gestión de Implementos Deportivos</t>
   </si>
   <si>
     <t xml:space="preserve">El sistema debe permitir el registro y control centralizado de los elementos deportivos del club. Se requiere una gestión eficiente de las solicitudes de préstamo y un seguimiento preciso de la disponibilidad de los recursos para los entrenamientos.
@@ -470,7 +470,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -494,7 +494,11 @@
     <xf borderId="7" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="8" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="8" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="9" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -562,11 +566,67 @@
     <xdr:ext cx="1028700" cy="1038225"/>
     <xdr:pic>
       <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>209550</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>1028700</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2238375" cy="9525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1685925</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>1028700</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2238375" cy="9525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
         <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
+        <a:blip cstate="print" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -585,96 +645,40 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>180975</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>971550</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2238375" cy="9525"/>
+      <xdr:rowOff>390525</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2305050" cy="647700"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1733550</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>390525</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1733550" cy="1295400"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1514475</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>971550</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2238375" cy="9525"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>142875</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>495300</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2305050" cy="647700"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1762125</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>419100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1733550" cy="1295400"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -707,7 +711,7 @@
     <xdr:ext cx="1028700" cy="1038225"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -735,7 +739,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -763,7 +767,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -819,7 +823,7 @@
     <xdr:ext cx="1733550" cy="1295400"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -852,7 +856,7 @@
     <xdr:ext cx="1028700" cy="1038225"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -880,7 +884,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -908,7 +912,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -964,7 +968,7 @@
     <xdr:ext cx="1733550" cy="1295400"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -992,7 +996,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1025,7 +1029,7 @@
     <xdr:ext cx="1028700" cy="1038225"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1053,7 +1057,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1081,7 +1085,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1109,7 +1113,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1165,7 +1169,7 @@
     <xdr:ext cx="1733550" cy="1295400"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1198,7 +1202,7 @@
     <xdr:ext cx="1028700" cy="1038225"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1226,7 +1230,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1254,7 +1258,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1282,7 +1286,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1338,7 +1342,7 @@
     <xdr:ext cx="1733550" cy="1295400"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1618,6 +1622,17 @@
       <c r="F6" s="9" t="s">
         <v>9</v>
       </c>
+      <c r="J6" s="11"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="12"/>
+      <c r="M6" s="12"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="12"/>
+      <c r="P6" s="12"/>
+      <c r="Q6" s="12"/>
+      <c r="R6" s="12"/>
+      <c r="S6" s="12"/>
+      <c r="T6" s="12"/>
     </row>
     <row r="7" ht="60.75" customHeight="1">
       <c r="B7" s="9" t="s">
@@ -1675,80 +1690,80 @@
   </cols>
   <sheetData>
     <row r="2" ht="89.25" customHeight="1">
-      <c r="B2" s="11"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="13" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="15" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" ht="21.75" customHeight="1">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="15" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="4" ht="358.5" customHeight="1">
-      <c r="B4" s="14">
+      <c r="B4" s="16">
         <v>3.0</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="17" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="5" ht="476.25" customHeight="1">
-      <c r="B5" s="17"/>
-      <c r="C5" s="18" t="s">
+      <c r="B5" s="19"/>
+      <c r="C5" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="12"/>
+      <c r="E5" s="14"/>
     </row>
     <row r="6" ht="106.5" customHeight="1">
-      <c r="B6" s="17"/>
-      <c r="C6" s="18" t="s">
+      <c r="B6" s="19"/>
+      <c r="C6" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="12"/>
+      <c r="E6" s="14"/>
     </row>
     <row r="7" ht="36.0" customHeight="1">
-      <c r="B7" s="17"/>
-      <c r="C7" s="18" t="s">
+      <c r="B7" s="19"/>
+      <c r="C7" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="21">
+      <c r="D7" s="23">
         <v>46136.0</v>
       </c>
-      <c r="E7" s="12"/>
+      <c r="E7" s="14"/>
     </row>
     <row r="8" ht="144.75" customHeight="1">
-      <c r="B8" s="17"/>
-      <c r="C8" s="22" t="s">
+      <c r="B8" s="19"/>
+      <c r="C8" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="23"/>
-      <c r="E8" s="12"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1776,80 +1791,80 @@
   </cols>
   <sheetData>
     <row r="2" ht="89.25" customHeight="1">
-      <c r="B2" s="11"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="13" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="15" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" ht="21.75" customHeight="1">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="15" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="4" ht="195.0" customHeight="1">
-      <c r="B4" s="14">
+      <c r="B4" s="16">
         <v>3.0</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="17" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="5" ht="246.75" customHeight="1">
-      <c r="B5" s="17"/>
-      <c r="C5" s="18" t="s">
+      <c r="B5" s="19"/>
+      <c r="C5" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="E5" s="12"/>
+      <c r="E5" s="14"/>
     </row>
     <row r="6" ht="106.5" customHeight="1">
-      <c r="B6" s="17"/>
-      <c r="C6" s="18" t="s">
+      <c r="B6" s="19"/>
+      <c r="C6" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="E6" s="12"/>
+      <c r="E6" s="14"/>
     </row>
     <row r="7" ht="36.0" customHeight="1">
-      <c r="B7" s="17"/>
-      <c r="C7" s="18" t="s">
+      <c r="B7" s="19"/>
+      <c r="C7" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="21">
+      <c r="D7" s="23">
         <v>46136.0</v>
       </c>
-      <c r="E7" s="12"/>
+      <c r="E7" s="14"/>
     </row>
     <row r="8" ht="144.75" customHeight="1">
-      <c r="B8" s="17"/>
-      <c r="C8" s="22" t="s">
+      <c r="B8" s="19"/>
+      <c r="C8" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="23"/>
-      <c r="E8" s="12"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1877,80 +1892,80 @@
   </cols>
   <sheetData>
     <row r="2" ht="89.25" customHeight="1">
-      <c r="B2" s="11"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="13" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="15" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" ht="21.75" customHeight="1">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="15" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="4" ht="296.25" customHeight="1">
-      <c r="B4" s="14">
+      <c r="B4" s="16">
         <v>4.0</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="17" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="5" ht="291.0" customHeight="1">
-      <c r="B5" s="17"/>
-      <c r="C5" s="18" t="s">
+      <c r="B5" s="19"/>
+      <c r="C5" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="E5" s="12"/>
+      <c r="E5" s="14"/>
     </row>
     <row r="6" ht="91.5" customHeight="1">
-      <c r="B6" s="17"/>
-      <c r="C6" s="18" t="s">
+      <c r="B6" s="19"/>
+      <c r="C6" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="E6" s="12"/>
+      <c r="E6" s="14"/>
     </row>
     <row r="7" ht="36.0" customHeight="1">
-      <c r="B7" s="17"/>
-      <c r="C7" s="18" t="s">
+      <c r="B7" s="19"/>
+      <c r="C7" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="21">
+      <c r="D7" s="23">
         <v>46136.0</v>
       </c>
-      <c r="E7" s="12"/>
+      <c r="E7" s="14"/>
     </row>
     <row r="8" ht="144.75" customHeight="1">
-      <c r="B8" s="17"/>
-      <c r="C8" s="22" t="s">
+      <c r="B8" s="19"/>
+      <c r="C8" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="23"/>
-      <c r="E8" s="12"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1978,80 +1993,80 @@
   </cols>
   <sheetData>
     <row r="2" ht="84.75" customHeight="1">
-      <c r="B2" s="11"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="25" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="E2" s="27" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" ht="21.75" customHeight="1">
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="D3" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="25" t="s">
+      <c r="E3" s="27" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="4" ht="263.25" customHeight="1">
-      <c r="B4" s="14">
+      <c r="B4" s="16">
         <v>2.0</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="17" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" ht="360.0" customHeight="1">
-      <c r="B5" s="17"/>
-      <c r="C5" s="18" t="s">
+      <c r="B5" s="19"/>
+      <c r="C5" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="E5" s="12"/>
+      <c r="E5" s="14"/>
     </row>
     <row r="6" ht="50.25" customHeight="1">
-      <c r="B6" s="17"/>
-      <c r="C6" s="18" t="s">
+      <c r="B6" s="19"/>
+      <c r="C6" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="E6" s="12"/>
+      <c r="E6" s="14"/>
     </row>
     <row r="7" ht="26.25" customHeight="1">
-      <c r="B7" s="17"/>
-      <c r="C7" s="18" t="s">
+      <c r="B7" s="19"/>
+      <c r="C7" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="21">
+      <c r="D7" s="23">
         <v>46136.0</v>
       </c>
-      <c r="E7" s="12"/>
+      <c r="E7" s="14"/>
     </row>
     <row r="8" ht="109.5" customHeight="1">
-      <c r="B8" s="17"/>
-      <c r="C8" s="22" t="s">
+      <c r="B8" s="19"/>
+      <c r="C8" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="D8" s="23"/>
-      <c r="E8" s="12"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2079,80 +2094,80 @@
   </cols>
   <sheetData>
     <row r="2" ht="84.75" customHeight="1">
-      <c r="B2" s="11"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="25" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="E2" s="27" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" ht="21.75" customHeight="1">
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="D3" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="25" t="s">
+      <c r="E3" s="27" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="4" ht="270.75" customHeight="1">
-      <c r="B4" s="14">
+      <c r="B4" s="16">
         <v>5.0</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="17" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" ht="283.5" customHeight="1">
-      <c r="B5" s="17"/>
-      <c r="C5" s="18" t="s">
+      <c r="B5" s="19"/>
+      <c r="C5" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="E5" s="12"/>
+      <c r="E5" s="14"/>
     </row>
     <row r="6" ht="50.25" customHeight="1">
-      <c r="B6" s="17"/>
-      <c r="C6" s="18" t="s">
+      <c r="B6" s="19"/>
+      <c r="C6" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="E6" s="12"/>
+      <c r="E6" s="14"/>
     </row>
     <row r="7" ht="26.25" customHeight="1">
-      <c r="B7" s="17"/>
-      <c r="C7" s="18" t="s">
+      <c r="B7" s="19"/>
+      <c r="C7" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="21">
+      <c r="D7" s="23">
         <v>46136.0</v>
       </c>
-      <c r="E7" s="12"/>
+      <c r="E7" s="14"/>
     </row>
     <row r="8" ht="109.5" customHeight="1">
-      <c r="B8" s="17"/>
-      <c r="C8" s="22" t="s">
+      <c r="B8" s="19"/>
+      <c r="C8" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="D8" s="23"/>
-      <c r="E8" s="12"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
V.4 partes interesadas en CheerClick Systems.
</commit_message>
<xml_diff>
--- a/Documentación/Trimestre I/Stakeholders_CheerClick_Systems.xlsx
+++ b/Documentación/Trimestre I/Stakeholders_CheerClick_Systems.xlsx
@@ -5,10 +5,11 @@
   <sheets>
     <sheet state="visible" name="Roles" sheetId="1" r:id="rId5"/>
     <sheet state="visible" name="Gestión de Usuarios" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Gestión de Horarios" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="Gestión de Rendimiento Deportiv" sheetId="4" r:id="rId8"/>
-    <sheet state="visible" name="Gestión de Elementos Deportivos" sheetId="5" r:id="rId9"/>
-    <sheet state="visible" name="Gestión de PQRS" sheetId="6" r:id="rId10"/>
+    <sheet state="visible" name="Gestión de Pagos" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="Gestión de Horarios" sheetId="4" r:id="rId8"/>
+    <sheet state="visible" name="Gestión de Rendimiento Deportiv" sheetId="5" r:id="rId9"/>
+    <sheet state="visible" name="Gestión de Implementos Deportiv" sheetId="6" r:id="rId10"/>
+    <sheet state="visible" name="Gestión de PQRS" sheetId="7" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -16,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="57">
   <si>
     <t>SISTEMA DE INFORMACIÓN CHEERCLICK SYSTEMS</t>
   </si>
@@ -100,21 +101,23 @@
     <t>Gestion de Horarios</t>
   </si>
   <si>
-    <t>Se requiere un módulo centralizado donde se gestione el ciclo de vida de los usuarios dentro de la plataforma, permitiendo el registro de nuevos atletas mediante un formato de captura de datos de contacto para establecer una comunicación efectiva y asegurar su correcta integración en la base de datos. Este componente debe garantizar la seguridad mediante un sistema de autenticación robusto y permitir la gestión de perfiles personalizados.. Asimismo, el sistema debe contemplar la administración de roles y el control de acceso robusto, asegurando que cada usuario interactúe únicamente con las funcionalidades permitidas según su nivel de autorización.
-De acuerdo con los estándares de recolección de información que mencionas, el formulario de registro base para los atletas debe contener los siguientes campos obligatorios:
+    <t xml:space="preserve">Se requiere un módulo centralizado donde se gestione el ciclo de vida de los usuarios dentro de la plataforma, permitiendo el registro de nuevos atletas mediante un formulario de captura de datos de contacto para establecer una comunicación efectiva y asegurar su correcta integración en la base de datos. Este componente debe garantizar la seguridad mediante un sistema de autenticación robusto y permitir la gestión de perfiles personalizados. Asimismo, el sistema debe contemplar la administración de roles y el control de acceso, asegurando que cada usuario interactúe únicamente con las funcionalidades permitidas según su rol.
+De acuerdo con las necesidades operativas del club, el formulario de registro base para los atletas debe contener los siguientes campos obligatorios:
 - Estado: Activo/Inactivo
-- Nombre completo
+- Nombre completo(personal)
 - Número y tipo de documento
-- Edad
-- Genero
-- Telefono
-- Telefono (Acudiente)
 - Fecha de nacimiento
-- Categoría
-- Email
+- Género
+- Teléfono (personal)
+- Nivel
+- Email  
 - Contraseña
+- Nombre de la EPS
 - Certificado de la EPS
-- Parentesco</t>
+- Parentesco
+- Nombre completo (contacto de emergencia)
+- Teléfono (contacto de emergencia)
+</t>
   </si>
   <si>
     <t>Alta</t>
@@ -123,35 +126,28 @@
     <t>Controles y restricciones o requerimientos no funcionales</t>
   </si>
   <si>
-    <t xml:space="preserve">RF-001 Registro de Usuarios
-El sistema debe permitir el registro de nuevos usuarios mediante el ingreso de información básica como nombre, correo electrónico, quedando la cuenta en estado pendiente hasta su validación por el administrador.
-RF - 002 Validación de Cuenta por Administrador
-El sistema debe permitir al administrador aceptar o rechazar las cuentas registradas por los usuarios antes de habilitar su acceso al sistema
-RF - 003 Notificación de Activación de Cuenta 
-El sistema debe notificar al usuario mediante correo electrónico ante el cambio de estado de su cuenta.
+    <t>RF-001 Home Page
+El sistema debe permitir al usuario desplazarse a las diferentes secciones de contenido (nosotros, servicios, niveles, horarios y contacto) mediante el menú de navegación superior. Asimismo, debe proporcionar accesos para iniciar sesión y realizar el proceso de registro para crear su cuenta.
+RF-002 Registro de Cuentas
+El sistema debe permitir que los interesados puedan crear su cuenta mediante el diligenciamiento de un formulario. Este formulario deberá solicitar información básica del atleta, incluyendo nombre completo, número de teléfono propio y del acudiente (junto con el parentesco), correo electrónico, fecha de nacimiento, género, nivel asignado, tipo y número de documento, así como el nombre de la EPS y certificado de afiliación a la misma. Una vez enviada la solicitud, ésta quedará en estado "Pendiente" hasta ser revisada y aprobada por el administrador. 
+RF - 003 Validación de Cuentas
+El sistema debe permitir al administrador visualizar la información de las cuentas registradas en el sistema antes de aceptar o rechazar el acceso de los usuarios al sistema. Durante el proceso de validación, el administrador podrá consultar la información suministrada y los documentos adjuntos para verificar su autenticidad y completitud.
 RF-004 Inicio de Sesión
-El sistema debe permitir a los usuarios autenticarse mediante correo electrónico y contraseña.
-RF- 005 Control de Intentos
-El sistema debe implementar autenticación mediante correo electrónico y contraseña, permitiendo un máximo de 3 intentos fallidos consecutivos antes de bloquear temporalmente la cuenta del usuario.
-RF- 006 Cambio de Contraseña
-El sistema debe permitir a los usuarios un cambio de contraseña en caso de que sea requerido.
-RF - 007 Actualizar Datos del Usuario
-El sistema debe permitir a los usuarios actualizar su información personal registrada
-RF - 008 Edición de Perfil de Usuario
- El sistema debe permitir al administrador, atleta y entrenador editar la información de su perfil personal, incluyendo datos de contacto, información de emergencia, preferencias de comunicación y contraseña, garantizando la seguridad y actualización correcta de los datos registrados en el sistema.
-RF- 009 Administración de Cuentas 
-El sistema debe permitir al administrador modificar, activar o desactivar cuentas de usuarios.
-RF- 010 Consulta y Registro de Estado de  Mensualidades
-El sistema debe permitir al administrador registrar y actualizar el estado de las mensualidades de los atletas indicando su respectivo estado con el envío de      notificaciones relacionadas.
-RF- 011 Cierre de Sesión
-El sistema debe permitir a los usuarios cerrar sesión de manera segura, finalizando su acceso a la plataforma.
-</t>
+El sistema debe permitir a los usuarios con rol de Administrador, Atleta y Entrenador autenticarse mediante correo electrónico y contraseña para acceder a las funcionalidades correspondientes a su perfil. El sistema deberá validar las credenciales ingresadas y verificar que la cuenta se encuentre activa antes de permitir el acceso.
+RF- 005 Cambio de Contraseña
+El sistema debe permitir a los usuarios con rol de Administrador, Atleta y Entrenador recuperar y cambiar su contraseña cuando sea requerido. Para ello, el usuario deberá proporcionar el correo electrónico asociado a su cuenta , validar su identidad mediante un código de verificación enviado al correo electrónico y establecer una nueva contraseña que cumpla con las políticas de seguridad definidas por la plataforma. 
+RF - 006 Edición de Perfil de Usuario
+El sistema debe permitir al administrador, atleta y entrenador editar la información de su perfil personal, incluyendo datos de contacto, información de emergencia, preferencias de comunicación y contraseña, garantizando la seguridad y actualización correcta de los datos registrados en el sistema.
+RF-007 Administración de Cuentas
+El sistema debe permitir exclusivamente al Administrador gestionar las cuentas de los usuarios con rol de Atleta y Entrenador, realizando acciones como consultar, modificar, activar o desactivar cuentas registradas en la plataforma. Los cambios efectuados deberán reflejarse de manera inmediata en el sistema para garantizar una administración adecuada de los accesos.
+RF- 008 Cierre de Sesión
+El sistema debe permitir a los usuarios cerrar sesión de manera segura, finalizando su acceso a la plataforma.</t>
   </si>
   <si>
     <t xml:space="preserve">Criterios de Aceptación </t>
   </si>
   <si>
-    <t>El sistema permite gestionar al usuario mediante un registro con validación de datos únicos y aprobación administrativa previa notificación por correo, permitiendo el acceso y la edición de perfiles únicamente a cuentas activas que superen una autenticación segura con bloqueo por intentos fallidos. Asimismo, debe garantizar el control de sesiones y permitir que el administrador actualice mensualidades con efecto inmediato, mientras el cliente consulta en tiempo real su historial de pagos y estados pendientes bajo un esquema estricto de seguridad y roles.</t>
+    <t xml:space="preserve">El sistema permite gestionar al usuario mediante un registro con validación de datos únicos y aprobación administrativa previa notificación por correo, permitiendo el acceso y la edición de perfiles únicamente a cuentas activas que superen una autenticación segura con bloqueo por intentos fallidos. </t>
   </si>
   <si>
     <t xml:space="preserve">Fecha de especificación </t>
@@ -161,6 +157,34 @@
      ( Dueño del proceso )                                         Usuarios participantes                                            Demás usuarios involucrados
      en la especificación                                             en la especificación
 </t>
+  </si>
+  <si>
+    <t>Gestion de Pagos</t>
+  </si>
+  <si>
+    <t>Se requiere un módulo centralizado para administrar los pagos dentro del sistema, permitiendo controlar el registro, consulta, validación y seguimiento de los pagos asociados a los atletas del club deportivo, con el fin de facilitar la gestión de mensualidades y pagos derivados de solicitudes de implementos previamente aprobadas.
+Este módulo deberá permitir el almacenamiento y validación de comprobantes digitales como soporte del pago, mantener el historial de transacciones realizadas y garantizar que cada usuario acceda únicamente a la información correspondiente según su rol dentro del sistema.
+De acuerdo con las necesidades operativas del club, el módulo debe contemplar el manejo de la siguiente información obligatoria para cada registro de pago:
+- Tipo de pago (Mensualidad / Implemento)                                                      - Plan asociado (Básico / Black / White) cuando aplique                                                           - Valor
+- Fecha de generación
+- Fecha de vencimiento
+- Fecha de pago
+- Método de pago
+- Comprobante de pago
+- Responsable del registro
+- Estado del pago (Pendiente / Pagado / Vencido / Rechazado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RF- 009 Consulta Historial de Pagos
+El sistema debe permitir al administrador y al atleta consultar la información de pagos registrados en el sistema, incluyendo mensualidades y pagos asociados a solicitudes de implementos deportivos.
+RF- 010 Validación de Pagos
+El sistema debe permitir al administrador validar y actualizar el estado de las mensualidades de los atletas (pagado, vencido y pendiente). Asimismo, debe permitir gestionar las solicitudes de implementos deportivos, ya sean aprobadas o rechazadas, enviando las notificaciones correspondientes en cada caso.
+RF - 011 Carga de Comprobante de Pago
+El sistema debe permitir al atleta cargar el comprobante de pago correspondiente a una mensualidad o a una compra de un implemento, adjuntando un archivo digital como evidencia del pago realizado. El comprobante será almacenado en el sistema para su posterior consulta y validación por parte del administrador.  
+</t>
+  </si>
+  <si>
+    <t>El sistema garantizará que la gestión de pagos e implementos sea segura, permitira que los usuarios carguen soportes digitales y consulten su historial personal, mientras que el administrador valida montos sean correctos y aprueba o rechaza solicitudes basándose en los comprobantes adjuntos. Para asegurar el control total, cada transacción debe registrar automáticamente la fecha, hora y usuario responsable, aplicando filtros por periodo o estado y enviando notificaciones automáticas al atleta y acudiente ante cualquier actualización de estado (pagado, pendiente, vencido, aprobado o rechazado), manteniendo siempre la integridad y claridad de los datos almacenados.</t>
   </si>
   <si>
     <t>Se requiere un módulo para la gestión de cronogramas donde el administrador configure las jornadas de entrenamiento y eventos para posteriormente generar una planificación de los horaios en la base de datos que permitirá establecer una organización eficiente del tiempo.
@@ -212,13 +236,19 @@
 El sistema debe permitir al entrenador evaluar y registrar el desempeño deportivo del atleta, incluyendo evaluaciones de desempeño, mientras que la asistencia será gestionada mediante los registros correspondientes del sistema.
 RF - 018 Consulta de Rendimiento Deportivo
 El sistema debe permitir a los usuarios autorizados consultar el rendimiento deportivo del atleta, incluyendo historial de evaluaciones y registro de asistencia.
-RF - 019  Actualización del Rendimiento Deportivo
-El sistema debe permitir al entrenador modificar registros de rendimiento deportivo, incluyendo evaluaciones y asistencia
+RF-019 Modificar Rendimiento Deportivo 
+El sistema debe permitir al Entrenador modificar los registros de rendimiento deportivo de los atletas, incluyendo evaluaciones de desempeño, con el fin de corregir o actualizar información previamente registrada. Las modificaciones realizadas deberán reflejarse inmediatamente en el historial del atleta.
 RF - 020 Inhabilitar  Registro de Rendimiento 
 El sistema debe permitir Inhabilitar registros de evaluaciones o asistencia en caso de errores o duplicados.
 RF-021 – Registro de Asistencia
- El sistema debe permitir al entrenador registrar la asistencia de los atletas a entrenamientos o eventos, filtrando por fecha o categoría y marcando el estado de cada participante (asistió, falta, justificado)
-RF - 022 Justificación de Inasistencia 
+El sistema debe permitir al entrenador registrar la asistencia de los atletas a entrenamientos o eventos, filtrando por fecha o categoría y marcando el estado de cada participante (asistió, falta, justificado)
+RF-022 Consultar Asistencia
+El sistema debe permitir a los usuarios autorizados consultar los registros de asistencia de los atletas a las sesiones de entrenamiento, mostrando el historial de participación y los estados de asistencia registrados por los entrenadores. 
+RF-023 Modificar Asistencia
+El sistema debe permitir al Entrenador modificar los registros de asistencia de los atletas cuando sea necesario corregir errores o actualizar información registrada incorrectamente. Las modificaciones realizadas deberán quedar reflejadas inmediatamente en el historial de asistencia del atleta. 
+RF-024 Inhabilitación de Asistencia 
+El sistema debe permitir al Entrenador inhabilitar registros de asistencia cuando se identifiquen errores, duplicidades o inconsistencias en la información registrada. Los registros inhabilitados deberán conservarse en el sistema para fines de auditoría e historial, pero no serán considerados en consultas, estadísticas o reportes activos. 
+RF - 025 Justificación de Inasistencia 
 El sistema debe permitir a los clientes justificar la ausencia antes o después de la sesión de entrenamiento programada en su horario.
 </t>
   </si>
@@ -231,44 +261,46 @@
 </t>
   </si>
   <si>
-    <t>Gestión de Elementos Deportivos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El sistema debe permitir el registro y control centralizado de los elementos deportivos del club. Se requiere una gestión eficiente de las solicitudes de préstamo y un seguimiento preciso de la disponibilidad de los recursos para los entrenamientos.
+    <t>Gestión de Implementos Deportivos</t>
+  </si>
+  <si>
+    <t>El sistema debe permitir el registro y control centralizado de los elementos deportivos del club. Se requiere una gestión eficiente de las solicitudes de préstamo y un seguimiento preciso de la disponibilidad de los recursos para los entrenamientos.
 El sistema debe gestionar los siguientes campos:
 Filtros de Busqueda
-Selección de pestaña: Implementos Deportivos/Productos Solicitados
+Selección de pestaña: Implementos Deportivos/Productos Solicitados(Adminitrador); Catalogo de Implementos, Mis solicitudes(Atleta)
 Nombre del Implemento
 Tipo de implemento
 Cantidad en stock
 Modificar Implemento deportivo
 Inhabilitar inplemento deportivo
 Precio del implemento
-Solicitud de pedido
+Talla
 Estado (Cliente: Pendiente/Cancelar/Listo para Entregar), (Administrador: Disponible/No Disponible/Pendiente/Rechazado/Aprobado)
-Nombre del solicitante
-Fecha de solicitud
-Fecha de entrega
-</t>
+Nombre del solicitante                                                                                                        Reseñas
+Fecha de solicitud</t>
   </si>
   <si>
     <t>Controles y Restrcciones o Requerimientos no Funcionales</t>
   </si>
   <si>
-    <t xml:space="preserve">RF - 023 Registro de Implementos Deportivos
+    <t xml:space="preserve">RF - 026 Registro de Implementos Deportivos
 El sistema debe permitir registrar los elementos deportivos, incluyendo nombre del elemento, tipo, precio, observaciones, cantidad disponible y estado.
-RF - 024 Solicitud de Implementos Deportivos
+RF - 027 Solicitud de Implementos Deportivos
 El sistema debe permitir que los clientes soliciten elementos deportivos para los entrenamientos y competencias.
-RF - 025 Aprobación de Solicitudes de Implementos
+RF - 028 Aprobación de Solicitudes de Implementos
 El sistema debe permitir al administrador aprobar o rechazar las solicitudes de implementos deportivos realizadas por los usuarios.
-RF - 026 Consultar Implementos deportivos
+RF - 029 Consultar Implementos deportivos
 El sistema debe permitir al administrador y a los atletas consultar el listado de implementos deportivos registrados, mostrando información detallada como nombre del implemento, cantidad disponible, estado, categoría.
-RF - 027 Consulta de Productos Solicitados 
+RF - 030 Consulta de Productos Solicitados 
 El sistema debe permitir al administrador y al cliente consultar el listado de productos solicitados, mostrando información detallada como el nombre del producto, cantidad, estado de la solicitud, fecha de registro y responsable. 
-RF - 028 Actualización de Implementos
+RF - 031 Actualización de Implementos
 El sistema debe permitir modificar la información de los implementos deportivos registrados.
-RF - 029 Cancelación  o Inhabilitación de Implementos
-El sistema debe permitir cancelar o inhabilitar implementos deportivos del sistema cuando el cliente quiera cancelarlo, ya no estén disponibles o se hayan discontinuado
+RF - 032 Cancelación  o Inhabilitación de Implementos
+El sistema debe permitir cancelar o inhabilitar implementos deportivos del sistema cuando el cliente quiera cancelarlo, ya no estén disponibles o se hayan discontinuado.                                                                                                                
+RF - 033 Confirmación de Recepción de Solicitud
+El sistema debe permitir al usuario marcar una solicitud de implementos deportivos como recibida cuando el pedido ya se encuentre en estado "Listo para entregar".
+RF - 034 Registro de Reseñas por el Usuario 
+El sistema debe permitir al usuario calificar con estrellas y dejar un comentario opcional sobre el producto recibido una vez que la solicitud se haya completado. 
 </t>
   </si>
   <si>
@@ -317,9 +349,7 @@
 El sistema debe permitir actualizar el estado y la información relacionada a una solicitud.
 RF- 034 Respuesta de PQRS
 El sistema debe permitir al administrador gestionar y responder las solicitudes registradas.
-RF-035 Notificación de Estado de PQRS
-El sistema debe notificar al usuario cuando su solicitud haya sido respondida.
-RF - 036 Inhabilitación de PQRS
+RF - 035 Inhabilitación de PQRS
 El sistema debe permitir al administrador inhabilitar solicitudes de PQRS cuando sea necesario.
 </t>
   </si>
@@ -470,7 +500,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -494,7 +524,11 @@
     <xf borderId="7" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="8" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="8" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="9" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -562,11 +596,67 @@
     <xdr:ext cx="1028700" cy="1038225"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>209550</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>1028700</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2238375" cy="9525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1685925</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>1028700</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2238375" cy="9525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -585,16 +675,16 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>180975</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>971550</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2238375" cy="9525"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
+      <xdr:rowOff>390525</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2305050" cy="647700"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -611,70 +701,14 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1514475</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>971550</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2238375" cy="9525"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>142875</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>495300</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2305050" cy="647700"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1762125</xdr:colOff>
+      <xdr:colOff>1733550</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>419100</xdr:rowOff>
+      <xdr:rowOff>390525</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1733550" cy="1295400"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -707,11 +741,67 @@
     <xdr:ext cx="1028700" cy="1038225"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>209550</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>1028700</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2238375" cy="9525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1685925</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>1028700</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2238375" cy="9525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -730,16 +820,16 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>180975</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>971550</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2238375" cy="9525"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
+      <xdr:rowOff>390525</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2305050" cy="647700"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -756,70 +846,14 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1514475</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>971550</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2238375" cy="9525"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>142875</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>495300</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2305050" cy="647700"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1762125</xdr:colOff>
+      <xdr:colOff>1733550</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>419100</xdr:rowOff>
+      <xdr:rowOff>390525</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1733550" cy="1295400"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -852,7 +886,7 @@
     <xdr:ext cx="1028700" cy="1038225"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -880,7 +914,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -929,14 +963,14 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>228600</xdr:colOff>
+      <xdr:colOff>142875</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>495300</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2019300" cy="571500"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+    <xdr:ext cx="2305050" cy="647700"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -959,44 +993,16 @@
       <xdr:col>3</xdr:col>
       <xdr:colOff>1762125</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>352425</xdr:rowOff>
+      <xdr:rowOff>419100</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1733550" cy="1295400"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip cstate="print" r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>4057650</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>971550</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2238375" cy="9525"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1018,158 +1024,158 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
+      <xdr:colOff>400050</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1028700" cy="1038225"/>
     <xdr:pic>
       <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>180975</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>971550</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2238375" cy="9525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1514475</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>971550</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2238375" cy="9525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>495300</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2019300" cy="571500"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1762125</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>352425</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1733550" cy="1295400"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
         <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>95250</xdr:colOff>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>4057650</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>590550</xdr:rowOff>
+      <xdr:rowOff>971550</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1676400</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>600075</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2238375" cy="9525"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>4314825</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>600075</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2238375" cy="9525"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>66675</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>66675</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2305050" cy="647700"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image5.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1847850</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>581025</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1733550" cy="1295400"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1198,7 +1204,7 @@
     <xdr:ext cx="1028700" cy="1038225"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1226,7 +1232,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1254,7 +1260,7 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1282,7 +1288,180 @@
     <xdr:ext cx="2238375" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2305050" cy="647700"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1847850</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>581025</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1733550" cy="1295400"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1028700" cy="1038225"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
         <xdr:cNvPr id="0" name="image3.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>590550</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2238375" cy="9525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1676400</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>600075</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2238375" cy="9525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>4314825</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>600075</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2238375" cy="9525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1310,7 +1489,7 @@
     <xdr:ext cx="1914525" cy="542925"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1338,7 +1517,7 @@
     <xdr:ext cx="1733550" cy="1295400"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Imagen"/>
+        <xdr:cNvPr id="0" name="image4.png" title="Imagen"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1618,6 +1797,17 @@
       <c r="F6" s="9" t="s">
         <v>9</v>
       </c>
+      <c r="J6" s="11"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="12"/>
+      <c r="M6" s="12"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="12"/>
+      <c r="P6" s="12"/>
+      <c r="Q6" s="12"/>
+      <c r="R6" s="12"/>
+      <c r="S6" s="12"/>
+      <c r="T6" s="12"/>
     </row>
     <row r="7" ht="60.75" customHeight="1">
       <c r="B7" s="9" t="s">
@@ -1675,80 +1865,80 @@
   </cols>
   <sheetData>
     <row r="2" ht="89.25" customHeight="1">
-      <c r="B2" s="11"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="13" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="15" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" ht="21.75" customHeight="1">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="15" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="4" ht="358.5" customHeight="1">
-      <c r="B4" s="14">
-        <v>3.0</v>
-      </c>
-      <c r="C4" s="15" t="s">
+    <row r="4" ht="345.0" customHeight="1">
+      <c r="B4" s="16">
+        <v>1.0</v>
+      </c>
+      <c r="C4" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="17" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="5" ht="476.25" customHeight="1">
-      <c r="B5" s="17"/>
-      <c r="C5" s="18" t="s">
+      <c r="B5" s="19"/>
+      <c r="C5" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="12"/>
+      <c r="E5" s="14"/>
     </row>
     <row r="6" ht="106.5" customHeight="1">
-      <c r="B6" s="17"/>
-      <c r="C6" s="18" t="s">
+      <c r="B6" s="19"/>
+      <c r="C6" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="12"/>
+      <c r="E6" s="14"/>
     </row>
     <row r="7" ht="36.0" customHeight="1">
-      <c r="B7" s="17"/>
-      <c r="C7" s="18" t="s">
+      <c r="B7" s="19"/>
+      <c r="C7" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="21">
-        <v>46136.0</v>
-      </c>
-      <c r="E7" s="12"/>
+      <c r="D7" s="23">
+        <v>46198.0</v>
+      </c>
+      <c r="E7" s="14"/>
     </row>
     <row r="8" ht="144.75" customHeight="1">
-      <c r="B8" s="17"/>
-      <c r="C8" s="22" t="s">
+      <c r="B8" s="19"/>
+      <c r="C8" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="23"/>
-      <c r="E8" s="12"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1776,80 +1966,80 @@
   </cols>
   <sheetData>
     <row r="2" ht="89.25" customHeight="1">
-      <c r="B2" s="11"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="13" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="15" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" ht="21.75" customHeight="1">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="15" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="4" ht="195.0" customHeight="1">
-      <c r="B4" s="14">
-        <v>3.0</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="D4" s="16" t="s">
+    <row r="4" ht="341.25" customHeight="1">
+      <c r="B4" s="16">
+        <v>2.0</v>
+      </c>
+      <c r="C4" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="D4" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="17" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" ht="246.75" customHeight="1">
-      <c r="B5" s="17"/>
-      <c r="C5" s="18" t="s">
+    <row r="5" ht="189.0" customHeight="1">
+      <c r="B5" s="19"/>
+      <c r="C5" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="E5" s="12"/>
+      <c r="D5" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="14"/>
     </row>
     <row r="6" ht="106.5" customHeight="1">
-      <c r="B6" s="17"/>
-      <c r="C6" s="18" t="s">
+      <c r="B6" s="19"/>
+      <c r="C6" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="E6" s="12"/>
+      <c r="D6" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" s="14"/>
     </row>
     <row r="7" ht="36.0" customHeight="1">
-      <c r="B7" s="17"/>
-      <c r="C7" s="18" t="s">
+      <c r="B7" s="19"/>
+      <c r="C7" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="21">
-        <v>46136.0</v>
-      </c>
-      <c r="E7" s="12"/>
+      <c r="D7" s="23">
+        <v>46198.0</v>
+      </c>
+      <c r="E7" s="14"/>
     </row>
     <row r="8" ht="144.75" customHeight="1">
-      <c r="B8" s="17"/>
-      <c r="C8" s="22" t="s">
+      <c r="B8" s="19"/>
+      <c r="C8" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="23"/>
-      <c r="E8" s="12"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1877,80 +2067,80 @@
   </cols>
   <sheetData>
     <row r="2" ht="89.25" customHeight="1">
-      <c r="B2" s="11"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="13" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="15" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" ht="21.75" customHeight="1">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="15" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="4" ht="296.25" customHeight="1">
-      <c r="B4" s="14">
-        <v>4.0</v>
-      </c>
-      <c r="C4" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" s="24" t="s">
+    <row r="4" ht="195.0" customHeight="1">
+      <c r="B4" s="16">
+        <v>3.0</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="17" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" ht="291.0" customHeight="1">
-      <c r="B5" s="17"/>
-      <c r="C5" s="18" t="s">
+    <row r="5" ht="246.75" customHeight="1">
+      <c r="B5" s="19"/>
+      <c r="C5" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="E5" s="12"/>
-    </row>
-    <row r="6" ht="91.5" customHeight="1">
-      <c r="B6" s="17"/>
-      <c r="C6" s="18" t="s">
+      <c r="E5" s="14"/>
+    </row>
+    <row r="6" ht="106.5" customHeight="1">
+      <c r="B6" s="19"/>
+      <c r="C6" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="E6" s="12"/>
+      <c r="E6" s="14"/>
     </row>
     <row r="7" ht="36.0" customHeight="1">
-      <c r="B7" s="17"/>
-      <c r="C7" s="18" t="s">
+      <c r="B7" s="19"/>
+      <c r="C7" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="21">
-        <v>46136.0</v>
-      </c>
-      <c r="E7" s="12"/>
+      <c r="D7" s="23">
+        <v>46198.0</v>
+      </c>
+      <c r="E7" s="14"/>
     </row>
     <row r="8" ht="144.75" customHeight="1">
-      <c r="B8" s="17"/>
-      <c r="C8" s="22" t="s">
+      <c r="B8" s="19"/>
+      <c r="C8" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="23"/>
-      <c r="E8" s="12"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1972,86 +2162,86 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="2" max="2" width="8.13"/>
-    <col customWidth="1" min="3" max="3" width="13.63"/>
-    <col customWidth="1" min="4" max="4" width="63.0"/>
-    <col customWidth="1" min="5" max="5" width="23.38"/>
+    <col customWidth="1" min="3" max="3" width="16.0"/>
+    <col customWidth="1" min="4" max="4" width="55.63"/>
+    <col customWidth="1" min="5" max="5" width="27.75"/>
   </cols>
   <sheetData>
-    <row r="2" ht="84.75" customHeight="1">
-      <c r="B2" s="11"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="25" t="s">
+    <row r="2" ht="89.25" customHeight="1">
+      <c r="B2" s="13"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="E2" s="15" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" ht="21.75" customHeight="1">
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="D3" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="25" t="s">
+      <c r="E3" s="15" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="4" ht="263.25" customHeight="1">
-      <c r="B4" s="14">
-        <v>2.0</v>
-      </c>
-      <c r="C4" s="18" t="s">
+    <row r="4" ht="259.5" customHeight="1">
+      <c r="B4" s="16">
+        <v>4.0</v>
+      </c>
+      <c r="C4" s="20" t="s">
         <v>41</v>
       </c>
       <c r="D4" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="E4" s="15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" ht="360.0" customHeight="1">
-      <c r="B5" s="17"/>
-      <c r="C5" s="18" t="s">
+      <c r="E4" s="17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" ht="393.0" customHeight="1">
+      <c r="B5" s="19"/>
+      <c r="C5" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="E5" s="14"/>
+    </row>
+    <row r="6" ht="91.5" customHeight="1">
+      <c r="B6" s="19"/>
+      <c r="C6" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="E5" s="12"/>
-    </row>
-    <row r="6" ht="50.25" customHeight="1">
-      <c r="B6" s="17"/>
-      <c r="C6" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="D6" s="20" t="s">
-        <v>46</v>
-      </c>
-      <c r="E6" s="12"/>
-    </row>
-    <row r="7" ht="26.25" customHeight="1">
-      <c r="B7" s="17"/>
-      <c r="C7" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="D7" s="21">
-        <v>46136.0</v>
-      </c>
-      <c r="E7" s="12"/>
-    </row>
-    <row r="8" ht="109.5" customHeight="1">
-      <c r="B8" s="17"/>
-      <c r="C8" s="22" t="s">
-        <v>48</v>
-      </c>
-      <c r="D8" s="23"/>
-      <c r="E8" s="12"/>
+      <c r="E6" s="14"/>
+    </row>
+    <row r="7" ht="36.0" customHeight="1">
+      <c r="B7" s="19"/>
+      <c r="C7" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="23">
+        <v>46198.0</v>
+      </c>
+      <c r="E7" s="14"/>
+    </row>
+    <row r="8" ht="144.75" customHeight="1">
+      <c r="B8" s="19"/>
+      <c r="C8" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="25"/>
+      <c r="E8" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2079,80 +2269,181 @@
   </cols>
   <sheetData>
     <row r="2" ht="84.75" customHeight="1">
-      <c r="B2" s="11"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="25" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="E2" s="27" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" ht="21.75" customHeight="1">
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="D3" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="25" t="s">
+      <c r="E3" s="27" t="s">
         <v>24</v>
       </c>
     </row>
+    <row r="4" ht="273.75" customHeight="1">
+      <c r="B4" s="16">
+        <v>5.0</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" s="28" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" ht="401.25" customHeight="1">
+      <c r="B5" s="19"/>
+      <c r="C5" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" s="14"/>
+    </row>
+    <row r="6" ht="50.25" customHeight="1">
+      <c r="B6" s="19"/>
+      <c r="C6" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="E6" s="14"/>
+    </row>
+    <row r="7" ht="26.25" customHeight="1">
+      <c r="B7" s="19"/>
+      <c r="C7" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="23">
+        <v>46198.0</v>
+      </c>
+      <c r="E7" s="14"/>
+    </row>
+    <row r="8" ht="109.5" customHeight="1">
+      <c r="B8" s="19"/>
+      <c r="C8" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="D8" s="25"/>
+      <c r="E8" s="14"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="C8:E8"/>
+  </mergeCells>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="2" max="2" width="8.13"/>
+    <col customWidth="1" min="3" max="3" width="13.63"/>
+    <col customWidth="1" min="4" max="4" width="63.0"/>
+    <col customWidth="1" min="5" max="5" width="23.38"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="84.75" customHeight="1">
+      <c r="B2" s="13"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" ht="21.75" customHeight="1">
+      <c r="B3" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" s="27" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="27" t="s">
+        <v>24</v>
+      </c>
+    </row>
     <row r="4" ht="270.75" customHeight="1">
-      <c r="B4" s="14">
-        <v>5.0</v>
-      </c>
-      <c r="C4" s="18" t="s">
+      <c r="B4" s="16">
+        <v>6.0</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" ht="258.75" customHeight="1">
+      <c r="B5" s="19"/>
+      <c r="C5" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>55</v>
+      </c>
+      <c r="E5" s="14"/>
+    </row>
+    <row r="6" ht="50.25" customHeight="1">
+      <c r="B6" s="19"/>
+      <c r="C6" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" ht="283.5" customHeight="1">
-      <c r="B5" s="17"/>
-      <c r="C5" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="D5" s="20" t="s">
+      <c r="D6" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" s="14"/>
+    </row>
+    <row r="7" ht="26.25" customHeight="1">
+      <c r="B7" s="19"/>
+      <c r="C7" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="E5" s="12"/>
-    </row>
-    <row r="6" ht="50.25" customHeight="1">
-      <c r="B6" s="17"/>
-      <c r="C6" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="D6" s="20" t="s">
+      <c r="D7" s="23">
+        <v>46198.0</v>
+      </c>
+      <c r="E7" s="14"/>
+    </row>
+    <row r="8" ht="109.5" customHeight="1">
+      <c r="B8" s="19"/>
+      <c r="C8" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="E6" s="12"/>
-    </row>
-    <row r="7" ht="26.25" customHeight="1">
-      <c r="B7" s="17"/>
-      <c r="C7" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="D7" s="21">
-        <v>46136.0</v>
-      </c>
-      <c r="E7" s="12"/>
-    </row>
-    <row r="8" ht="109.5" customHeight="1">
-      <c r="B8" s="17"/>
-      <c r="C8" s="22" t="s">
-        <v>48</v>
-      </c>
-      <c r="D8" s="23"/>
-      <c r="E8" s="12"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>